<commit_message>
chore: update competitor dealer report 周一 2-26-05
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,29 +12572,29 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12685,12 +12685,12 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12845,12 +12845,12 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,29 +12860,29 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,29 +12988,29 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13192,17 +13192,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,29 +13372,29 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,29 +14044,29 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,29 +14108,29 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,29 +14396,29 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14637,12 +14637,12 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14669,12 +14669,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,14 +14716,14 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
@@ -14733,12 +14733,12 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,29 +14844,29 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14957,12 +14957,12 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -15117,12 +15117,12 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -15149,12 +15149,12 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -15245,12 +15245,12 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -15277,12 +15277,12 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,29 +15388,29 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15523,7 +15523,7 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -15533,12 +15533,12 @@
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15592,17 +15592,17 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15656,17 +15656,17 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-05-25
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -12296,17 +12296,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,29 +12316,29 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12493,12 +12493,12 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,29 +12700,29 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,29 +12764,29 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -12909,12 +12909,12 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13192,17 +13192,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,29 +13276,29 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,29 +13404,29 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13581,12 +13581,12 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,29 +13628,29 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13741,12 +13741,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,29 +13756,29 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -13933,12 +13933,12 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,29 +13948,29 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,29 +14076,29 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14189,12 +14189,12 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -14509,12 +14509,12 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14541,12 +14541,12 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,29 +14716,29 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,29 +14908,29 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,14 +15452,14 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
@@ -15469,12 +15469,12 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 周一 2-26-06
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -12269,12 +12269,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,29 +12284,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -12333,12 +12333,12 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12493,12 +12493,12 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -12589,12 +12589,12 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,29 +12764,29 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,29 +12796,29 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,29 +12892,29 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -13005,12 +13005,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -13101,12 +13101,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13197,12 +13197,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,29 +13244,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,29 +13276,29 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,29 +13628,29 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,29 +13820,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,29 +13948,29 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,29 +14140,29 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,29 +14172,29 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,29 +14236,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -14285,12 +14285,12 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -14317,12 +14317,12 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14541,12 +14541,12 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14637,12 +14637,12 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,29 +14908,29 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -14989,12 +14989,12 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -15021,12 +15021,12 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,29 +15452,29 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-06-01
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -12269,12 +12269,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12296,17 +12296,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,29 +12540,29 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,29 +12572,29 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,29 +12796,29 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,29 +12892,29 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13197,12 +13197,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,29 +13244,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,29 +13532,29 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,29 +13692,29 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,29 +13820,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,29 +14140,29 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,29 +14172,29 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,29 +14236,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14317,12 +14317,12 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -14541,12 +14541,12 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14605,12 +14605,12 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14669,12 +14669,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,29 +14780,29 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,29 +14876,29 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14989,12 +14989,12 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -15117,12 +15117,12 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,29 +15260,29 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-06-08
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,14 +12284,14 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -12301,12 +12301,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,29 +12316,29 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,29 +12444,29 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,29 +12924,29 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,14 +13180,14 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -13197,12 +13197,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -13261,12 +13261,12 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13485,12 +13485,12 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,29 +13788,29 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,29 +13980,29 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,29 +14140,29 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14221,12 +14221,12 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14509,12 +14509,12 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,29 +14588,29 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,29 +15004,29 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,29 +15036,29 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,14 +15100,14 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
@@ -15117,12 +15117,12 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,29 +15164,29 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,29 +15324,29 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15592,17 +15592,17 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15688,17 +15688,17 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-06-15
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,29 +12284,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -12525,12 +12525,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,29 +13116,29 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13165,12 +13165,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,14 +13180,14 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -13197,12 +13197,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,29 +13372,29 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,29 +13788,29 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,29 +13820,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,29 +13980,29 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,29 +14428,29 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14509,12 +14509,12 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,29 +14812,29 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,29 +15036,29 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,29 +15100,29 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,29 +15164,29 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,29 +15292,29 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15437,12 +15437,12 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15720,17 +15720,17 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-06-16
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12296,17 +12296,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -12749,12 +12749,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,29 +13020,29 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,29 +13116,29 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -13192,17 +13192,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,29 +13372,29 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,29 +13500,29 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,14 +13756,14 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
@@ -13773,12 +13773,12 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,29 +13820,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13933,12 +13933,12 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,29 +14268,29 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,29 +14396,29 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,29 +14428,29 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -14573,12 +14573,12 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,29 +14588,29 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -14797,12 +14797,12 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,29 +14812,29 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,14 +15164,14 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
@@ -15181,12 +15181,12 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,29 +15260,29 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,29 +15292,29 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -15405,12 +15405,12 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -15437,12 +15437,12 @@
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15469,12 +15469,12 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -15528,17 +15528,17 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,7 +15651,7 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
@@ -15661,12 +15661,12 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-06-22
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,29 +12284,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,29 +12444,29 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -12781,12 +12781,12 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,29 +12828,29 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,29 +12860,29 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -13192,17 +13192,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13453,12 +13453,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,29 +13564,29 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,29 +13596,29 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,29 +13628,29 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,29 +13852,29 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14157,12 +14157,12 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,29 +14204,29 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -14253,12 +14253,12 @@
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,29 +14268,29 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -14541,12 +14541,12 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -14573,12 +14573,12 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,14 +14652,14 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
@@ -14669,12 +14669,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,29 +14716,29 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14957,12 +14957,12 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,29 +15324,29 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -15373,12 +15373,12 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,29 +15452,29 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-06-29
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -12301,12 +12301,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,29 +12508,29 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,29 +12860,29 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -13192,17 +13192,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,29 +13212,29 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,29 +13244,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,29 +13276,29 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -13357,12 +13357,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,29 +13564,29 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,29 +13596,29 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -13741,12 +13741,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,29 +13788,29 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14061,12 +14061,12 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14157,12 +14157,12 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,29 +14236,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,29 +14268,29 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,29 +14652,29 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,29 +14716,29 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14925,12 +14925,12 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,29 +15324,29 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -15373,12 +15373,12 @@
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-06
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -12296,17 +12296,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,29 +12476,29 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,29 +12508,29 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -12589,12 +12589,12 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,29 +12700,29 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,29 +12796,29 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -12909,12 +12909,12 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,29 +13180,29 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,29 +13212,29 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,29 +13244,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,29 +13276,29 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -13325,12 +13325,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,29 +13340,29 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,29 +13468,29 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,29 +13788,29 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -14093,12 +14093,12 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -14189,12 +14189,12 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,29 +14236,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,29 +14268,29 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -15053,12 +15053,12 @@
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,29 +15164,29 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15624,17 +15624,17 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-13
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11523,7 +11523,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11535,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11550,7 +11550,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,29 +12284,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,14 +12476,14 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -12493,12 +12493,12 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,29 +12668,29 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,29 +12700,29 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,29 +12796,29 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,29 +12892,29 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,29 +13180,29 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,29 +13244,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,29 +13340,29 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -13421,12 +13421,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,29 +13468,29 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -13549,12 +13549,12 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,29 +13628,29 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13741,12 +13741,12 @@
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -13837,12 +13837,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,29 +13852,29 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13901,12 +13901,12 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14061,12 +14061,12 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -14093,12 +14093,12 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14472,17 +14472,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14600,17 +14600,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,29 +14620,29 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14669,12 +14669,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14797,12 +14797,12 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,29 +15164,29 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15469,12 +15469,12 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -15523,7 +15523,7 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
@@ -15533,12 +15533,12 @@
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15560,17 +15560,17 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15592,17 +15592,17 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-14
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10806,7 +10806,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10821,7 +10821,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,29 +12284,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,29 +12348,29 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,7 +12572,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12584,17 +12584,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,29 +12668,29 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,29 +12892,29 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -12973,12 +12973,12 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,7 +13116,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -13128,17 +13128,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,7 +13148,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -13160,17 +13160,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,29 +13180,29 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,14 +13244,14 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -13261,12 +13261,12 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13453,12 +13453,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,29 +13628,29 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13773,12 +13773,12 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,7 +13820,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -13832,17 +13832,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,29 +13852,29 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,7 +14012,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14024,17 +14024,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,29 +14460,29 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,29 +14588,29 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,29 +14620,29 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -14669,12 +14669,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -14728,17 +14728,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14824,17 +14824,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,29 +15196,29 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,29 +15228,29 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -15405,12 +15405,12 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15469,12 +15469,12 @@
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15560,17 +15560,17 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15624,17 +15624,17 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-15
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10887,7 +10887,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11211,7 +11211,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11238,7 +11238,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11253,7 +11253,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12264,17 +12264,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -12296,17 +12296,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,29 +12348,29 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12456,17 +12456,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12520,17 +12520,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,29 +12540,29 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,29 +12572,29 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -12968,17 +12968,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13069,12 +13069,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,29 +13116,29 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,14 +13148,14 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -13165,12 +13165,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,29 +13180,29 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -13320,17 +13320,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,29 +13628,29 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,14 +13820,14 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -13837,12 +13837,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -13896,17 +13896,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,7 +13948,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -13960,17 +13960,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -13992,17 +13992,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,29 +14012,29 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,29 +14460,29 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14568,17 +14568,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,29 +14588,29 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,29 +14716,29 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,7 +14780,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14792,17 +14792,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -14829,12 +14829,12 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14861,12 +14861,12 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,7 +15132,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -15144,17 +15144,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,29 +15196,29 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,29 +15228,29 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15309,12 +15309,12 @@
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,7 +15356,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -15368,17 +15368,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15587,22 +15587,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15619,22 +15619,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15651,22 +15651,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15688,17 +15688,17 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15720,17 +15720,17 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-20
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10794,7 +10794,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10848,7 +10848,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10929,7 +10929,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10941,7 +10941,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11076,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11091,7 +11091,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11103,7 +11103,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11292,7 +11292,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11307,7 +11307,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11319,7 +11319,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11334,7 +11334,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11415,7 +11415,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11427,7 +11427,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11589,7 +11589,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11604,7 +11604,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11616,7 +11616,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11631,7 +11631,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11643,7 +11643,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11928,7 +11928,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12269,12 +12269,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12284,7 +12284,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -12296,17 +12296,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12316,7 +12316,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -12328,17 +12328,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12360,17 +12360,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12380,7 +12380,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -12392,17 +12392,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12412,7 +12412,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -12424,17 +12424,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12444,29 +12444,29 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12476,7 +12476,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -12488,17 +12488,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12508,7 +12508,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12525,12 +12525,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12540,29 +12540,29 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12572,29 +12572,29 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12604,7 +12604,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -12616,17 +12616,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12636,7 +12636,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -12648,17 +12648,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12668,7 +12668,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12680,17 +12680,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12700,7 +12700,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12712,17 +12712,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12732,7 +12732,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -12744,17 +12744,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12764,7 +12764,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -12776,17 +12776,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12796,7 +12796,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -12808,17 +12808,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12828,7 +12828,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -12840,17 +12840,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12860,7 +12860,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -12872,17 +12872,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -12904,17 +12904,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12924,7 +12924,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12936,17 +12936,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12956,7 +12956,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -12973,12 +12973,12 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12988,7 +12988,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13000,17 +13000,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -13032,17 +13032,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13052,7 +13052,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -13064,17 +13064,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13084,7 +13084,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13096,17 +13096,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13116,29 +13116,29 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13148,29 +13148,29 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13180,7 +13180,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13192,17 +13192,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13212,7 +13212,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -13224,17 +13224,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13256,17 +13256,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13276,7 +13276,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -13288,17 +13288,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13308,7 +13308,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -13325,12 +13325,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13340,7 +13340,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13384,17 +13384,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13404,7 +13404,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -13416,17 +13416,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13436,7 +13436,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13448,17 +13448,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13480,17 +13480,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -13512,17 +13512,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -13544,17 +13544,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -13576,17 +13576,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13608,17 +13608,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -13640,17 +13640,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13672,17 +13672,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13704,17 +13704,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13724,7 +13724,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13736,17 +13736,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13756,7 +13756,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13768,17 +13768,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13788,7 +13788,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13800,17 +13800,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13820,29 +13820,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13852,7 +13852,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -13864,17 +13864,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13884,7 +13884,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -13901,12 +13901,12 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13916,7 +13916,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13928,17 +13928,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13948,29 +13948,29 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13980,7 +13980,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13997,12 +13997,12 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14012,29 +14012,29 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14044,7 +14044,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14056,17 +14056,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14076,7 +14076,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14088,17 +14088,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14108,7 +14108,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14120,17 +14120,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14140,7 +14140,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -14152,17 +14152,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14172,7 +14172,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -14184,17 +14184,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14204,7 +14204,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14216,17 +14216,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14236,7 +14236,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14248,17 +14248,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14268,7 +14268,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14280,17 +14280,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14300,7 +14300,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -14312,17 +14312,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14332,7 +14332,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14344,17 +14344,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14364,7 +14364,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -14376,17 +14376,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14396,7 +14396,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -14408,17 +14408,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14428,7 +14428,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14440,17 +14440,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14460,7 +14460,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -14477,12 +14477,12 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -14504,17 +14504,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14524,7 +14524,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14536,17 +14536,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14573,12 +14573,12 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14605,12 +14605,12 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14620,7 +14620,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14632,17 +14632,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14652,7 +14652,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -14664,17 +14664,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14684,7 +14684,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14696,17 +14696,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14716,29 +14716,29 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14748,7 +14748,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14760,17 +14760,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14780,29 +14780,29 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -14829,12 +14829,12 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14844,7 +14844,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -14856,17 +14856,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14876,7 +14876,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -14888,17 +14888,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14908,7 +14908,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14920,17 +14920,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14940,7 +14940,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -14952,17 +14952,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14972,7 +14972,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -14984,17 +14984,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15004,7 +15004,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -15016,17 +15016,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -15048,17 +15048,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15068,7 +15068,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -15080,17 +15080,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -15112,17 +15112,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15132,29 +15132,29 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15164,7 +15164,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -15176,17 +15176,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15196,7 +15196,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -15208,17 +15208,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15228,7 +15228,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -15240,17 +15240,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15260,7 +15260,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -15272,17 +15272,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15292,7 +15292,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15304,17 +15304,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15324,7 +15324,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -15336,17 +15336,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15356,29 +15356,29 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15388,7 +15388,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -15400,17 +15400,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15420,7 +15420,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -15432,17 +15432,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15452,7 +15452,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -15464,17 +15464,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15484,7 +15484,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -15523,22 +15523,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15555,22 +15555,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15592,17 +15592,17 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15683,22 +15683,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15715,22 +15715,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-27
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="新增网点（19家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="减少网点（58家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="变更明细（111条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10848,7 +10848,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10956,7 +10956,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10971,7 +10971,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10998,7 +10998,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11388,7 +11388,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11550,7 +11550,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11565,7 +11565,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11658,7 +11658,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11673,7 +11673,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11685,7 +11685,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11700,7 +11700,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11928,7 +11928,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11943,7 +11943,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11955,7 +11955,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12301,22 +12301,22 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12326,7 +12326,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -12338,17 +12338,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12358,29 +12358,29 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12390,7 +12390,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -12402,17 +12402,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12422,7 +12422,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -12434,17 +12434,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12454,7 +12454,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -12471,12 +12471,12 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12486,7 +12486,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12498,17 +12498,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12518,7 +12518,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -12530,17 +12530,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12567,12 +12567,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12582,29 +12582,29 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>新疆</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -12626,17 +12626,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12646,7 +12646,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -12658,17 +12658,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -12695,12 +12695,12 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12710,7 +12710,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12722,17 +12722,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12742,7 +12742,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -12759,12 +12759,12 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12774,7 +12774,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12786,17 +12786,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12806,7 +12806,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -12818,17 +12818,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12838,7 +12838,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -12850,17 +12850,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12870,7 +12870,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12882,17 +12882,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12902,7 +12902,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -12914,17 +12914,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12934,7 +12934,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -12946,17 +12946,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12966,7 +12966,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -12983,12 +12983,12 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12998,29 +12998,29 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -13030,7 +13030,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -13074,17 +13074,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13094,7 +13094,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13106,17 +13106,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -13138,17 +13138,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13158,7 +13158,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13170,17 +13170,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13190,7 +13190,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13202,17 +13202,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13222,7 +13222,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13234,17 +13234,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13254,29 +13254,29 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13298,17 +13298,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13318,7 +13318,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13330,17 +13330,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13350,7 +13350,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -13362,17 +13362,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13382,7 +13382,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13394,17 +13394,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13414,7 +13414,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13426,17 +13426,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13446,29 +13446,29 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13478,7 +13478,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13490,17 +13490,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13510,7 +13510,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13522,17 +13522,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13542,7 +13542,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -13554,17 +13554,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13574,7 +13574,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -13586,17 +13586,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13606,7 +13606,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -13618,17 +13618,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -13650,17 +13650,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13670,7 +13670,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -13682,17 +13682,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13702,7 +13702,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13714,17 +13714,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13734,7 +13734,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -13746,17 +13746,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13766,7 +13766,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -13778,17 +13778,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13798,7 +13798,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13810,17 +13810,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13830,7 +13830,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -13842,17 +13842,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13862,7 +13862,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13874,17 +13874,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13894,7 +13894,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13906,17 +13906,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13926,7 +13926,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13938,17 +13938,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13958,29 +13958,29 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13990,7 +13990,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14002,17 +14002,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -14022,7 +14022,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14039,12 +14039,12 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -14054,7 +14054,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14066,17 +14066,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14086,29 +14086,29 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14118,7 +14118,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -14130,17 +14130,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14162,17 +14162,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14182,7 +14182,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14194,17 +14194,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14214,7 +14214,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14231,12 +14231,12 @@
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14246,7 +14246,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14258,17 +14258,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14278,7 +14278,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -14290,17 +14290,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14310,7 +14310,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14322,17 +14322,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14354,17 +14354,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14374,7 +14374,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -14386,17 +14386,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14423,12 +14423,12 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14438,7 +14438,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -14450,17 +14450,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14470,7 +14470,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14482,17 +14482,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14502,7 +14502,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14514,17 +14514,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14534,7 +14534,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -14546,17 +14546,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14566,7 +14566,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14578,17 +14578,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14598,29 +14598,29 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>鸿蒙智行</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>华为智能生活馆•杭州黄龙国际中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14642,17 +14642,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14662,7 +14662,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -14674,17 +14674,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14694,7 +14694,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14706,17 +14706,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14726,14 +14726,14 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
@@ -14743,12 +14743,12 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14758,7 +14758,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14775,12 +14775,12 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14790,7 +14790,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14802,17 +14802,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14822,7 +14822,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14834,17 +14834,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14854,7 +14854,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14866,17 +14866,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14886,29 +14886,29 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -14930,17 +14930,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14950,29 +14950,29 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>华为智能生活馆•杭州黄龙国际中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14982,7 +14982,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>浙江省杭州市西湖区学院路77号黄龙万科中心AB楼1F → 浙江省杭州市西湖区翠苑街道学院路77号1楼华为</t>
         </is>
       </c>
     </row>
@@ -14994,17 +14994,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -15014,7 +15014,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -15026,17 +15026,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -15046,29 +15046,29 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -15078,7 +15078,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -15090,17 +15090,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15110,7 +15110,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -15122,17 +15122,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -15154,17 +15154,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -15186,17 +15186,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -15218,17 +15218,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15238,7 +15238,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15250,17 +15250,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15270,7 +15270,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -15282,17 +15282,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15302,7 +15302,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15314,17 +15314,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15334,7 +15334,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -15346,17 +15346,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15378,17 +15378,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15398,29 +15398,29 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>鸿蒙智行</t>
         </is>
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>新疆</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>鸿蒙智行尚界用户中心•阿克苏大欣汽车城</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15430,7 +15430,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏悦诚汽车销售有限公司1#2号厅 → 新疆维吾尔自治区阿克苏地区温宿县温宿镇幸福路与建业街交汇处阿克苏尚锦汽车销售有限公司1#2号厅</t>
         </is>
       </c>
     </row>
@@ -15442,17 +15442,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -15474,17 +15474,17 @@
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15506,17 +15506,17 @@
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15526,7 +15526,7 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -15570,17 +15570,17 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15597,22 +15597,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15666,17 +15666,17 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15693,22 +15693,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -15725,22 +15725,22 @@
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -15757,22 +15757,22 @@
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-07-30
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -851,10 +851,10 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>1480</v>
+        <v>1479</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1479</v>
+        <v>1478</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>-1</v>
@@ -872,10 +872,10 @@
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>8606</v>
+        <v>8605</v>
       </c>
       <c r="C19" s="1" t="n">
-        <v>8566</v>
+        <v>8565</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>-40</v>
@@ -9892,10 +9892,10 @@
         </is>
       </c>
       <c r="C428" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D428" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E428" s="2" t="n">
         <v>0</v>
@@ -11199,7 +11199,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11241,7 +11241,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11916,7 +11916,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12225,17 +12225,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12257,17 +12257,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12289,17 +12289,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,29 +12309,29 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -12353,17 +12353,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12486,12 +12486,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12545,17 +12545,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -12641,17 +12641,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12673,17 +12673,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -12865,17 +12865,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,29 +12917,29 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -12993,17 +12993,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,29 +13013,29 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13089,17 +13089,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13126,12 +13126,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -13185,17 +13185,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,29 +13205,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13281,17 +13281,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,29 +13301,29 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13382,12 +13382,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,29 +13397,29 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13441,17 +13441,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13473,17 +13473,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13537,17 +13537,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -13606,12 +13606,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13633,17 +13633,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,29 +13685,29 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,29 +13781,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -13825,17 +13825,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13921,17 +13921,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14113,17 +14113,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14209,17 +14209,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -14433,17 +14433,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14497,17 +14497,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,7 +14517,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14529,17 +14529,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14561,17 +14561,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -14625,17 +14625,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,7 +14645,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14657,17 +14657,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -14721,17 +14721,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,14 +14773,14 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
@@ -14790,12 +14790,12 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14854,12 +14854,12 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -15078,12 +15078,12 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,29 +15125,29 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15233,17 +15233,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15452,22 +15452,22 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15484,22 +15484,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15516,22 +15516,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15548,22 +15548,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15580,22 +15580,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15617,17 +15617,17 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-08-03
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（17家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（57家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（109条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="新增网点（17家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="减少网点（57家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="变更明细（109条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11199,7 +11199,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11241,7 +11241,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11388,7 +11388,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11415,7 +11415,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11496,7 +11496,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11916,7 +11916,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12225,17 +12225,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -12257,17 +12257,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -12289,17 +12289,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -12321,17 +12321,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -12358,12 +12358,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -12481,17 +12481,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12545,17 +12545,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -12582,12 +12582,12 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12641,17 +12641,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -12673,17 +12673,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12838,12 +12838,12 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12865,17 +12865,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -12929,17 +12929,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -12993,17 +12993,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13025,17 +13025,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -13089,17 +13089,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13126,12 +13126,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -13185,17 +13185,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,29 +13205,29 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,29 +13237,29 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13281,17 +13281,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,29 +13301,29 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13414,12 +13414,12 @@
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13441,17 +13441,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13473,17 +13473,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13537,17 +13537,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13606,12 +13606,12 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -13633,17 +13633,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,29 +13685,29 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13793,17 +13793,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -13825,17 +13825,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -13921,17 +13921,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14113,17 +14113,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,29 +14165,29 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -14209,17 +14209,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -14246,12 +14246,12 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14433,17 +14433,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -14497,17 +14497,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,29 +14517,29 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -14561,17 +14561,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14598,12 +14598,12 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -14625,17 +14625,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,7 +14645,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14657,17 +14657,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,29 +14677,29 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14721,17 +14721,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -14785,17 +14785,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -14817,17 +14817,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -14950,12 +14950,12 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -15110,12 +15110,12 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,29 +15125,29 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -15233,17 +15233,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -15452,22 +15452,22 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15484,22 +15484,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15516,22 +15516,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15553,17 +15553,17 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15580,22 +15580,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15612,22 +15612,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-08-07
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="新增网点（17家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="减少网点（57家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="变更明细（109条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（17家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（57家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（109条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10767,7 +10767,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -11496,7 +11496,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -12230,12 +12230,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,29 +12245,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -12289,17 +12289,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,29 +12309,29 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -12353,17 +12353,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -12481,17 +12481,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -12545,17 +12545,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -12641,17 +12641,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -12673,17 +12673,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12865,17 +12865,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -12929,17 +12929,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,29 +12981,29 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -13025,17 +13025,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13089,17 +13089,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -13121,17 +13121,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -13185,17 +13185,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -13217,17 +13217,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,29 +13269,29 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13318,12 +13318,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -13350,12 +13350,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13409,17 +13409,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13446,12 +13446,12 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -13473,17 +13473,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,29 +13525,29 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13601,17 +13601,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -13633,17 +13633,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13697,17 +13697,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,14 +13749,14 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
@@ -13766,12 +13766,12 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -13793,17 +13793,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13825,17 +13825,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,29 +13845,29 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -13921,17 +13921,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14118,12 +14118,12 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14209,17 +14209,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14246,12 +14246,12 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14406,12 +14406,12 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14433,17 +14433,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -14497,17 +14497,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,7 +14517,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -14529,17 +14529,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,29 +14549,29 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14593,17 +14593,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,29 +14613,29 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,14 +14645,14 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
@@ -14662,12 +14662,12 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -14721,17 +14721,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14785,17 +14785,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14822,12 +14822,12 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -15137,17 +15137,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -15233,17 +15233,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15452,22 +15452,22 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15484,22 +15484,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15612,22 +15612,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-08-10
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="新增网点（17家）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="减少网点（57家）" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="变更明细（109条）" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="品牌总量对比" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="省级网点对比" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="新增网点（17家）" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="减少网点（57家）" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="变更明细（109条）" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11496,7 +11496,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11916,7 +11916,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -12230,12 +12230,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,29 +12245,29 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -12289,17 +12289,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,29 +12309,29 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -12353,17 +12353,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -12481,17 +12481,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -12545,17 +12545,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,29 +12629,29 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,29 +12661,29 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12865,17 +12865,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -12929,17 +12929,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -12966,12 +12966,12 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -12993,17 +12993,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -13030,12 +13030,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13089,17 +13089,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -13121,17 +13121,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13185,17 +13185,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13217,17 +13217,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,29 +13269,29 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -13313,17 +13313,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13409,17 +13409,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13446,12 +13446,12 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13473,17 +13473,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,29 +13525,29 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13601,17 +13601,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13633,17 +13633,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13697,17 +13697,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13766,12 +13766,12 @@
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13793,17 +13793,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -13825,17 +13825,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,29 +13909,29 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14118,12 +14118,12 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,29 +14197,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -14278,12 +14278,12 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -14433,17 +14433,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -14497,17 +14497,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,29 +14517,29 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14561,17 +14561,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -14593,17 +14593,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -14625,17 +14625,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,29 +14645,29 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -14817,17 +14817,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -15137,17 +15137,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -15233,17 +15233,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15452,22 +15452,22 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15484,22 +15484,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15516,22 +15516,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15548,22 +15548,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15580,22 +15580,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-08-17
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10794,7 +10794,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10875,7 +10875,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥肥西县合肥肥西旭辉CMALL</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>合肥市肥西县翡翠路与派河大道交口西侧旭辉CMALL3号门中庭</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11064,7 +11064,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11091,7 +11091,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11496,7 +11496,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -12225,17 +12225,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -12257,17 +12257,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -12289,17 +12289,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12321,17 +12321,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -12353,17 +12353,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -12481,17 +12481,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,29 +12533,29 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,29 +12629,29 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,29 +12661,29 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -12865,17 +12865,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -12934,12 +12934,12 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -12993,17 +12993,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13030,12 +13030,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,29 +13077,29 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -13121,17 +13121,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,29 +13173,29 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13217,17 +13217,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -13281,17 +13281,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -13313,17 +13313,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -13409,17 +13409,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -13441,17 +13441,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13473,17 +13473,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -13537,17 +13537,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -13601,17 +13601,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13633,17 +13633,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13697,17 +13697,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,14 +13781,14 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
@@ -13798,12 +13798,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -13825,17 +13825,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,29 +13909,29 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14113,17 +14113,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,29 +14197,29 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14433,17 +14433,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14497,17 +14497,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,29 +14517,29 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -14566,12 +14566,12 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -14593,17 +14593,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -14625,17 +14625,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,7 +14645,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14657,17 +14657,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -14721,17 +14721,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14758,12 +14758,12 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -14785,17 +14785,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14817,17 +14817,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15137,17 +15137,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -15233,17 +15233,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -15366,12 +15366,12 @@
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15457,17 +15457,17 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15484,22 +15484,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15516,22 +15516,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15580,22 +15580,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15612,22 +15612,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-08-24
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10767,7 +10767,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -12225,17 +12225,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -12257,17 +12257,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,29 +12277,29 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -12321,17 +12321,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,29 +12341,29 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,7 +12469,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -12481,17 +12481,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,29 +12533,29 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -12673,17 +12673,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,29 +12853,29 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -12929,17 +12929,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12993,17 +12993,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -13025,17 +13025,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,29 +13077,29 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -13121,17 +13121,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,29 +13173,29 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -13217,17 +13217,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -13281,17 +13281,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13313,17 +13313,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -13409,17 +13409,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13446,12 +13446,12 @@
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,29 +13461,29 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -13537,17 +13537,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -13601,17 +13601,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,7 +13621,7 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13633,17 +13633,17 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13697,17 +13697,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,29 +13781,29 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -13825,17 +13825,17 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -13921,17 +13921,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -13958,12 +13958,12 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -14113,17 +14113,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14209,17 +14209,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14433,17 +14433,17 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -14497,17 +14497,17 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,7 +14517,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -14529,17 +14529,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -14561,17 +14561,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14593,17 +14593,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -14625,17 +14625,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,7 +14645,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14657,17 +14657,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -14721,17 +14721,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14785,17 +14785,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14817,17 +14817,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14918,12 +14918,12 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -15137,17 +15137,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -15238,12 +15238,12 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15452,22 +15452,22 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15489,17 +15489,17 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15521,17 +15521,17 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15548,22 +15548,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15612,22 +15612,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-08-31
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10767,7 +10767,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -11064,7 +11064,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
+          <t>小米汽车广东深圳坪山区益田假日世界</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -11079,7 +11079,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
+          <t>六联社区深汕路(坪山段)168号中庭</t>
         </is>
       </c>
     </row>
@@ -11091,7 +11091,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>小米汽车广东深圳坪山区益田假日世界</t>
+          <t>小米汽车广东深圳宝安区满京华·满纷天地</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -11106,7 +11106,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>六联社区深汕路(坪山段)168号中庭</t>
+          <t>小米汽车(深圳满京华·满纷天地城市展厅)</t>
         </is>
       </c>
     </row>
@@ -11199,7 +11199,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11241,7 +11241,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11280,7 +11280,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州昆山招商花园城</t>
+          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -11295,7 +11295,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>萧林中路666号招商花园城一楼中庭</t>
+          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
+          <t>小米汽车江苏苏州昆山招商花园城</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -11322,7 +11322,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
+          <t>萧林中路666号招商花园城一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11334,7 +11334,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏苏州虎丘区绿宝广场</t>
+          <t>小米汽车江苏苏州张家港张家港曼巴特广场</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -11349,7 +11349,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>江苏省苏州市长江路436号绿宝广场一楼南中庭</t>
+          <t>江苏省苏州市张家港市杨舍镇河西路88号曼巴特购物中心一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11388,7 +11388,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11415,7 +11415,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11496,7 +11496,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州乐清市现代广场</t>
+          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>城南街道宴海西路777号L1-008</t>
+          <t>永定路1188号万达广场中庭</t>
         </is>
       </c>
     </row>
@@ -11523,7 +11523,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>小米汽车浙江温州龙湾区温州龙湾万达</t>
+          <t>小米汽车浙江温州乐清市现代广场</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -11538,7 +11538,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>永定路1188号万达广场中庭</t>
+          <t>城南街道宴海西路777号L1-008</t>
         </is>
       </c>
     </row>
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11874,7 +11874,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>厦门海上世界城市中心店</t>
+          <t>厦门建发众骋4S中心</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -11889,7 +11889,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市湖里区远航路77号</t>
+          <t>福建省厦门市集美区岩兴路89号</t>
         </is>
       </c>
     </row>
@@ -11901,7 +11901,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>厦门建发众骋4S中心</t>
+          <t>厦门海上世界城市中心店</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -11916,7 +11916,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>福建省厦门市集美区岩兴路89号</t>
+          <t>福建省厦门市湖里区远航路77号</t>
         </is>
       </c>
     </row>
@@ -12225,17 +12225,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -12257,17 +12257,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,29 +12277,29 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -12321,17 +12321,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,29 +12341,29 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,29 +12469,29 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12545,17 +12545,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,29 +12629,29 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -12673,17 +12673,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -12705,17 +12705,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,29 +12853,29 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,7 +12885,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
@@ -12897,17 +12897,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12929,17 +12929,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -12998,12 +12998,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -13025,17 +13025,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -13089,17 +13089,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
@@ -13121,17 +13121,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -13190,12 +13190,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13217,17 +13217,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -13281,17 +13281,17 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13313,17 +13313,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -13409,17 +13409,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13441,17 +13441,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,29 +13461,29 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -13505,17 +13505,17 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -13537,17 +13537,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -13601,17 +13601,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,29 +13621,29 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -13697,17 +13697,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
@@ -13793,17 +13793,17 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,29 +13813,29 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -13921,17 +13921,17 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14081,17 +14081,17 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14113,17 +14113,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -14209,17 +14209,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,7 +14357,7 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -14369,17 +14369,17 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,29 +14421,29 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,29 +14485,29 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,7 +14517,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -14529,17 +14529,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -14561,17 +14561,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14593,17 +14593,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -14625,17 +14625,17 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,7 +14645,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14657,17 +14657,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -14721,17 +14721,17 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -14785,17 +14785,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14817,17 +14817,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -14982,12 +14982,12 @@
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
@@ -15142,12 +15142,12 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -15233,17 +15233,17 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15452,22 +15452,22 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲销售中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉白沙洲大道销售中心</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15484,22 +15484,22 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车武汉白沙洲销售中心</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车武汉白沙洲大道销售中心</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -15516,22 +15516,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15580,22 +15580,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15612,22 +15612,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update competitor dealer report 2026-09-07
</commit_message>
<xml_diff>
--- a/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
+++ b/report/downloads/reports/网点变化对比报告_20260504_vs_20260511.xlsx
@@ -10767,7 +10767,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京丰台区丰科万达</t>
+          <t>小米汽车北京朝阳区东坝万达</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -10782,7 +10782,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>丰科万达一层中庭</t>
+          <t>东坝万达广场一层中庭</t>
         </is>
       </c>
     </row>
@@ -10794,7 +10794,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京朝阳区东坝万达</t>
+          <t>小米汽车北京昌平区昌平悦荟</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>东坝万达广场一层中庭</t>
+          <t>昌平悦荟一层中庭</t>
         </is>
       </c>
     </row>
@@ -10821,7 +10821,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>小米汽车北京昌平区昌平悦荟</t>
+          <t>小米汽车北京丰台区丰科万达</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -10836,7 +10836,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>昌平悦荟一层中庭</t>
+          <t>丰科万达一层中庭</t>
         </is>
       </c>
     </row>
@@ -10902,7 +10902,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
+          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
+          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>小米汽车安徽合肥长丰县北城世纪金源</t>
+          <t>小米汽车安徽合肥庐阳区庐阳万象汇</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>安徽省合肥市长丰县双墩镇蒙城北路与阜阳北路交口购物中心内A座一层A1号门老庙黄金旁</t>
+          <t>安徽省合肥市庐阳区庐阳万象汇3号门连廊</t>
         </is>
       </c>
     </row>
@@ -11199,7 +11199,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
+          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11214,7 +11214,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
+          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11226,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>小米汽车江苏常州天宁区常州九洲新世界</t>
+          <t>小米汽车江苏常州天宁区天宁吾悦广场</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -11241,7 +11241,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>兰陵北路999号九洲新世界广场一楼中庭</t>
+          <t>江苏省常州市天宁区东方西路10号天宁吾悦广场L1龙门厅</t>
         </is>
       </c>
     </row>
@@ -11388,7 +11388,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
+          <t>小米汽车河南郑州二七区二七万达</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
+          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
         </is>
       </c>
     </row>
@@ -11415,7 +11415,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>小米汽车河南郑州二七区二七万达</t>
+          <t>小米汽车河南郑州金水区郑州银泰inPARK</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>大学南路8号二七万达广场一楼小米汽车展台</t>
+          <t>河南郑州市金水区（郑东）龙湖金融岛郑州银泰inpark D区1F层D-L1009小米之家旁</t>
         </is>
       </c>
     </row>
@@ -11577,7 +11577,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆大渡口区大渡口万象汇</t>
+          <t>小米汽车重庆巴南区巴南万达</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -11592,7 +11592,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>重庆大渡口区万象汇LG层中庭</t>
+          <t>重庆巴南万达1F中庭</t>
         </is>
       </c>
     </row>
@@ -11604,7 +11604,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆巴南区巴南万达</t>
+          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -11619,7 +11619,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>重庆巴南万达1F中庭</t>
+          <t>龙湖礼嘉天街A馆-1F-中庭</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11631,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>小米汽车重庆两江新区龙湖礼嘉天街</t>
+          <t>小米汽车重庆大渡口区大渡口万象汇</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -11646,7 +11646,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>龙湖礼嘉天街A馆-1F-中庭</t>
+          <t>重庆大渡口区万象汇LG层中庭</t>
         </is>
       </c>
     </row>
@@ -12225,17 +12225,17 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
+          <t>小鹏汽车黄山屯光大道销售服务中心</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -12245,7 +12245,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
+          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
         </is>
       </c>
     </row>
@@ -12262,12 +12262,12 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车潮州潮汕路销售服务中心</t>
+          <t>小鹏汽车佛山南庄销售服务中心</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
+          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
         </is>
       </c>
     </row>
@@ -12289,17 +12289,17 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
+          <t>小鹏汽车武汉东西湖销售服务中心</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
+          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
         </is>
       </c>
     </row>
@@ -12321,17 +12321,17 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州龙湾销售服务中心</t>
+          <t>小鹏汽车常德大道销售中心</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -12341,7 +12341,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
+          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
         </is>
       </c>
     </row>
@@ -12353,17 +12353,17 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德销售服务中心</t>
+          <t>小鹏汽车靖江吾悦广场销售展厅</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -12373,7 +12373,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
+          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
         </is>
       </c>
     </row>
@@ -12385,17 +12385,17 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
+          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -12405,7 +12405,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
+          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
         </is>
       </c>
     </row>
@@ -12417,17 +12417,17 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
+          <t>小鹏汽车潮州潮汕路销售服务中心</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -12437,7 +12437,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
+          <t>广东省潮州市潮汕公路乌洋路段 → 广东省潮安区潮汕公路乌洋路段</t>
         </is>
       </c>
     </row>
@@ -12449,17 +12449,17 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
+          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -12469,29 +12469,29 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
+          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>上汽奥迪湘潭腾飞用户中心</t>
+          <t>小鹏汽车成都龙潭寺销售服务中心</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
+          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
         </is>
       </c>
     </row>
@@ -12513,17 +12513,17 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
+          <t>小鹏汽车柳州东环路销售服务中心</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -12533,7 +12533,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
+          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12545,17 +12545,17 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
+          <t>小鹏汽车河源大道销售服务中心</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -12565,7 +12565,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
+          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车许昌许州北路销售服务中心</t>
+          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -12597,7 +12597,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
+          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
         </is>
       </c>
     </row>
@@ -12609,17 +12609,17 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>天津</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
+          <t>小鹏汽车天津北辰双江道销售服务中心</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
+          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
         </is>
       </c>
     </row>
@@ -12641,17 +12641,17 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车济南经十西路销售服务中心</t>
+          <t>小鹏汽车台州路桥服务中心</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -12661,7 +12661,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
+          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
         </is>
       </c>
     </row>
@@ -12673,17 +12673,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
+          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -12693,29 +12693,29 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
+          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奔驰</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>天津</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车天津北辰双江道销售服务中心</t>
+          <t>广安华星锦业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -12725,7 +12725,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>天津市北辰区双街镇庞大汽贸园原五菱骏宝店展厅 → 天津市北辰区双街镇庞大汽贸园原五菱宝骏店展厅</t>
+          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
         </is>
       </c>
     </row>
@@ -12737,17 +12737,17 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车珠海上冲销售服务中心</t>
+          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -12757,7 +12757,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
+          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
         </is>
       </c>
     </row>
@@ -12769,17 +12769,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车河源大道销售服务中心</t>
+          <t>小鹏汽车临沂北京东路销售服务中心</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>河源市源城区河源大道南中国石油南侧250米 → 河源市源城区河源大道南中裕丰田汽车旁</t>
+          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
         </is>
       </c>
     </row>
@@ -12801,17 +12801,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山海八路销售服务中心</t>
+          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -12821,7 +12821,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
+          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -12833,17 +12833,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
+          <t>小鹏汽车南通东方汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
+          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
         </is>
       </c>
     </row>
@@ -12865,17 +12865,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
+          <t>小鹏汽车玉溪太极路销售服务中心</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -12885,29 +12885,29 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
+          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山南庄销售服务中心</t>
+          <t>上汽奥迪湘潭腾飞用户中心</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -12917,7 +12917,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>佛山市禅城区南庄镇醒群社村工业区5号 → 广东省佛山市禅城区南庄镇樵乐路(吉利大道西)杜村工业区5号</t>
+          <t>湖南省湘潭市雨湖区九华大道8号 → 湖南省湘潭市雨湖区潭州大道8号</t>
         </is>
       </c>
     </row>
@@ -12929,17 +12929,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车百色大旺路销售服务中心</t>
+          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
+          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
         </is>
       </c>
     </row>
@@ -12961,17 +12961,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
+          <t>小鹏汽车重庆万州沙龙路销售服务中心</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -12981,7 +12981,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
+          <t>重庆市万州区双河口街道沙龙路三段2243号（妇幼保健院路口） → 重庆市万州区沙龙路三段2243号</t>
         </is>
       </c>
     </row>
@@ -12993,17 +12993,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车德阳八角销售服务中心</t>
+          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
+          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
         </is>
       </c>
     </row>
@@ -13025,17 +13025,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
+          <t>小鹏汽车郑州东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -13045,7 +13045,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
+          <t>河南自贸试验区郑州片区（经开）航海路北、第七大街东1388号 → 河南省郑州市管城回族区航海路北第七大街东1386号小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13057,17 +13057,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
+          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -13077,7 +13077,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
+          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
         </is>
       </c>
     </row>
@@ -13089,17 +13089,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>广西</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳龙岗联创销售服务中心</t>
+          <t>小鹏汽车百色大旺路销售服务中心</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>广东省深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技园1栋厂房A、BA201 → 深圳市龙岗区南湾街道下李朗社区布澜路21号联创科技1栋厂房A、B区A101A201</t>
+          <t>广西百色市右江区大旺路14号 → 大旺路14号</t>
         </is>
       </c>
     </row>
@@ -13121,17 +13121,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车黄山屯光大道销售服务中心</t>
+          <t>小鹏汽车西安浐灞销售服务中心</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -13141,7 +13141,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>安徽省黄山市屯溪区屯光大道36号 小鹏汽车 → 安徽省黄山市屯溪区屯光大道36号</t>
+          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
         </is>
       </c>
     </row>
@@ -13153,17 +13153,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
+          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -13173,7 +13173,7 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
+          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
         </is>
       </c>
     </row>
@@ -13185,17 +13185,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车眉山眉州大道销售服务中心</t>
+          <t>小鹏汽车驻马店金龙汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
+          <t>开源大道东金龙科技园区16号厂房自西到东1-8跨，自北到南1-4跨 → 开源大道与兴业大道交叉口金龙科技园西门北侧1-4跨</t>
         </is>
       </c>
     </row>
@@ -13217,17 +13217,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口南海大道销售服务中心</t>
+          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
+          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
         </is>
       </c>
     </row>
@@ -13249,17 +13249,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车广州广汕路销售服务中心</t>
+          <t>小鹏汽车昆明车行天下服务中心</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
+          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
         </is>
       </c>
     </row>
@@ -13286,12 +13286,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山三水销售服务中心</t>
+          <t>小鹏汽车阳江泰基汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -13301,7 +13301,7 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
+          <t>广东省阳江市新江东路侧泰基新能源汽车城1号地块 → 阳江市新江东路侧泰基新能源汽车城1号地块</t>
         </is>
       </c>
     </row>
@@ -13313,17 +13313,17 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴柯桥销售服务中心</t>
+          <t>小鹏汽车威海金蚂蚁汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -13333,7 +13333,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
+          <t>山东省威海市环翠区温泉西路119号32号 → 威海市环翠区温泉西路119-7号14号展厅</t>
         </is>
       </c>
     </row>
@@ -13345,17 +13345,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车云浮环市西路销售服务中心</t>
+          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -13365,7 +13365,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
+          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
         </is>
       </c>
     </row>
@@ -13377,17 +13377,17 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京清河安宁庄销售服务中心</t>
+          <t>小鹏汽车汕尾大道销售服务中心</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -13397,7 +13397,7 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>北京市海淀区清河街道西三旗桥向南600米路西小鹏汽车 → 北京市海淀区安宁庄后街南1号C区1层1301号</t>
+          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
         </is>
       </c>
     </row>
@@ -13409,17 +13409,17 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>广西</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车柳州东环路销售服务中心</t>
+          <t>小鹏汽车德阳八角销售服务中心</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>广西壮族自治区柳州市城中区河东街道东环大道155号南方电网鹿山充电站 → 广西壮族自治区柳州市城中区河东街道东环大道157号南方电网鹿山充电站小鹏汽车</t>
+          <t>四川省德阳市八角工业园区柳江街1幢 → 德阳市旌阳区八角工业园区柳江街1号（老车管所旁）</t>
         </is>
       </c>
     </row>
@@ -13441,17 +13441,17 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车嘉兴汽车商贸园销售服务中心</t>
+          <t>小鹏汽车佛山顺德销售服务中心</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -13461,7 +13461,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>浙江省嘉兴市南湖区东栅街道汽车商贸园文贤路与南江路交叉口 → 嘉兴市南湖区广益路汽车商贸园文贤路与南江路交叉口小鹏汽车</t>
+          <t>广东省佛山市顺德区大良街道横八路21号(小鹏汽车佛山顺德交付中心) → 佛山市顺德区大良街道新松社区105国道新松路段6号</t>
         </is>
       </c>
     </row>
@@ -13473,17 +13473,17 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
+          <t>小鹏汽车佛山三水销售服务中心</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
+          <t>佛山市三水区云东海街道南丰大道26号C座首层八号商铺 → 广东省佛山市三水区云东海街道南丰大道26号C座首层</t>
         </is>
       </c>
     </row>
@@ -13510,12 +13510,12 @@
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州路桥服务中心</t>
+          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>浙江省台州市路桥区新安南街760号 → 浙江省台州市路桥区新安南街766号</t>
+          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
         </is>
       </c>
     </row>
@@ -13537,17 +13537,17 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车余姚东部汽车城销售服务中心</t>
+          <t>小鹏汽车珠海上冲销售服务中心</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>浙江省宁波市余姚市凤山街道同光村东江汽车城8号 → 浙江省余姚市凤山街道同光村余丈路2号（319省道）</t>
+          <t>广东省珠海市香洲区凤山街道华威路115号厂房3栋一楼101 → 广东省珠海市香洲区华威路115号</t>
         </is>
       </c>
     </row>
@@ -13569,17 +13569,17 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车常德大道销售中心</t>
+          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -13589,7 +13589,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>武陵区常德大道1888号 → 湖南省常德市武陵区东江街道新安社区启明中路(武陵工业新区101-01号)</t>
+          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
         </is>
       </c>
     </row>
@@ -13601,17 +13601,17 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车诸暨北二环销售服务中心</t>
+          <t>小鹏汽车邯郸时代汽车广场销售服务中心</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -13621,29 +13621,29 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
+          <t>河北省邯郸市经开区时代汽车广场内B馆西南侧 → 河北省邯郸市经开区时代汽车城内B馆西南侧</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
+          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>李渔路888号 → 城北街道世贸购物广场</t>
+          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
         </is>
       </c>
     </row>
@@ -13665,17 +13665,17 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车武汉东西湖销售服务中心</t>
+          <t>小鹏汽车温州龙湾销售服务中心</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>武汉市东西湖区张柏路10号附23 → 武汉市东西湖区金银湖街环湖中路东、田园东路北A-3栋1层1室</t>
+          <t>浙江省温州市龙湾区高一路178号 → 浙江省温州市经济技术开发区高一路178号</t>
         </is>
       </c>
     </row>
@@ -13697,17 +13697,17 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>湖南</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车上饶月亮湾汽车城销售服务中心</t>
+          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -13717,7 +13717,7 @@
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>江西省上饶市经济技术开发区三清山西大道58号１单元103号104号 → 江西省上饶经济技术开发区三清山西大道58号１单元103号104号</t>
+          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
         </is>
       </c>
     </row>
@@ -13729,17 +13729,17 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南通东方汽车城销售服务中心</t>
+          <t>小鹏汽车杭州石祥东路销售服务中心</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>江苏省南通市开发区吉达路11号 → 南通市开发区东方汽车城吉达路11号</t>
+          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
         </is>
       </c>
     </row>
@@ -13761,17 +13761,17 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车通辽瑞丰汽贸园销售服务中心</t>
+          <t>小鹏汽车泸州纳溪经开区汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -13781,7 +13781,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>内蒙古自治区通辽市经济技术开发区创业大道与阿其玛大街交汇处东南110米 → 内蒙古自治区通辽市经济技术开发区创业大道与兴工大街交汇处以东</t>
+          <t>四川省泸州市纳溪区东升街道蓝安路三段19号小鹏汽车 → 四川	省泸州市纳溪区蓝安路三段兴业路1号</t>
         </is>
       </c>
     </row>
@@ -13798,12 +13798,12 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州石祥东路销售服务中心</t>
+          <t>小鹏汽车义乌北苑销售服务中心</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -13813,29 +13813,29 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>浙江省杭州市拱墅区东石祥东路1726号 → 浙江省杭州市拱墅区石祥东路1726号</t>
+          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>奔驰</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>广安华星锦业汽车销售服务有限公司</t>
+          <t>小鹏汽车宜兴融达汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -13845,7 +13845,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>枣山物流商贸园区物流大道A线 → 建民中路179号1幢</t>
+          <t>无锡市宜兴市经济开发区融达汽车城西氿大道90号 → 宜兴市经济开发区融达汽车城西氿大道90号</t>
         </is>
       </c>
     </row>
@@ -13857,17 +13857,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车揭阳荣通销售服务中心</t>
+          <t>小鹏汽车西昌航天大道销售服务中心</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -13877,7 +13877,7 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
+          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
         </is>
       </c>
     </row>
@@ -13889,17 +13889,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车兰州安宁汽车城销售服务中心</t>
+          <t>小鹏汽车巴中经开区汽贸园销售服务中心</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>甘肃省兰州市安宁区北滨河西路兰州金岛智鹏汽车销售服务有限公司 → 甘肃省兰州市安宁区北滨河西路1746号安宁汽车城15号</t>
+          <t>四川省巴中市兴文区龙兴大道金华泰汽车产业园 → 四川省巴中市兴文区龙兴大道金华泰汽车产业园小鹏销售服务中心</t>
         </is>
       </c>
     </row>
@@ -13926,12 +13926,12 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海宁城北销售服务中心</t>
+          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -13941,7 +13941,7 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
+          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
         </is>
       </c>
     </row>
@@ -13953,17 +13953,17 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>内蒙古</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宁波江北销售服务中心</t>
+          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
+          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -13985,17 +13985,17 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车湖州蜀山路销售服务中心</t>
+          <t>小鹏汽车成都空港销售服务中心</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -14005,7 +14005,7 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
+          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
         </is>
       </c>
     </row>
@@ -14017,17 +14017,17 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
+          <t>小鹏汽车南昌青山湖销售服务中心</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
+          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
         </is>
       </c>
     </row>
@@ -14049,17 +14049,17 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>北京</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京成寿寺销售服务中心</t>
+          <t>小鹏汽车眉山眉州大道销售服务中心</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -14069,29 +14069,29 @@
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
+          <t>四川省眉山市东坡区眉州大道西五段 → 四川省眉山市东坡区尚义镇经济开发区新区兴业路南段6号小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明世博园销售服务中心</t>
+          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
+          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
         </is>
       </c>
     </row>
@@ -14113,17 +14113,17 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车遂宁物流港汽车城销售服务中心</t>
+          <t>小鹏汽车重庆礼嘉服务中心</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>遂宁市物流港物流大道858-888号 → 四川省遂宁市遂宁高新区物流港物流大道858-888号</t>
+          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
         </is>
       </c>
     </row>
@@ -14145,17 +14145,17 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西昌航天大道销售服务中心</t>
+          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -14165,7 +14165,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>凉山州西昌市航天大道三段60号 → 四川省西昌市安宁镇新区5幢一层5号</t>
+          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
         </is>
       </c>
     </row>
@@ -14177,17 +14177,17 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>安徽</t>
+          <t>北京</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
+          <t>小鹏汽车北京亦庄销售服务中心</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -14197,7 +14197,7 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
+          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
         </is>
       </c>
     </row>
@@ -14209,17 +14209,17 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车义乌北苑销售服务中心</t>
+          <t>小鹏汽车广州广汕路销售服务中心</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -14229,7 +14229,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>浙江省金华市义乌市北苑路300号 → 浙江省义乌市 北苑路 300 号 （十亿客创业园内）</t>
+          <t>广州市天河区广汕二路119号102房 → 广州市天河广汕二路119号102房</t>
         </is>
       </c>
     </row>
@@ -14241,17 +14241,17 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沂北京东路销售服务中心</t>
+          <t>小鹏汽车宁波江北销售服务中心</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>山东省临沂市河东区温泉路与北京东路交汇处远通汽车超市小鹏汽车 → 临沂市河东区北京东路与温泉路交汇远通汽车超市院内</t>
+          <t>浙江宁波江北区中官新路555号5号-1 宁波小鹏交付中心 → 浙江省宁波市江北区中官新路555号</t>
         </is>
       </c>
     </row>
@@ -14273,17 +14273,17 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都锦江服务中心</t>
+          <t>小鹏汽车海口南海大道销售服务中心</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -14293,7 +14293,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
+          <t>海南省海口市龙华区南海大道115号 → 海南省海口市龙华区南海大道115号福德汽车城小鹏汽车</t>
         </is>
       </c>
     </row>
@@ -14305,17 +14305,17 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车宝鸡高新汽车城销售服务中心</t>
+          <t>小鹏汽车揭阳荣通销售服务中心</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>宝鸡市渭滨区高新十二路19号 → 陕西省宝鸡市高新开发区八鱼镇十二路19号（东风本田4S店右侧）</t>
+          <t>广东省揭阳市榕城区东石北路荣通汽车城 → 广东省揭阳市榕城区环市北路与新河路交界处荣通汽车城内</t>
         </is>
       </c>
     </row>
@@ -14337,17 +14337,17 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车娄底湘阳街汽车城销售服务中心</t>
+          <t>小鹏汽车佛山海八路销售服务中心</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -14357,29 +14357,29 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>娄底市娄星区湘阳街与檀香路交汇处 → 娄底市娄星区檀香路与湘阳街交汇处</t>
+          <t>广东省佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车 → 佛山市南海区桂城街道海八西路15号华南世纪车城2栋首层2-101/106 小鹏汽车</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>贵州</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车扬州国际汽车城服务中心</t>
+          <t>贵州华星名仕汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
+          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
         </is>
       </c>
     </row>
@@ -14401,17 +14401,17 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车汕尾大道销售服务中心</t>
+          <t>小鹏汽车绍兴柯桥销售服务中心</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -14421,29 +14421,29 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>广东省汕尾市城区红草镇海汕公路汕尾市君乐汽车销售服务有限公司 → 广东省汕尾市城区红草镇埔边工业区（原汕尾君乐4S店）</t>
+          <t>浙江省绍兴市柯桥区金柯桥大道2827号 → 绍兴市柯桥区金柯桥大道2827号</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>重庆市迪威奥迪汽车销售服务有限公司</t>
+          <t>小鹏汽车大理丰赢汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -14453,7 +14453,7 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>重庆市万州区江南新区联合坝机场路595号 → 重庆市万州区江南新区联合坝机场路591号</t>
+          <t>云南省大理白族自治州大理市凤仪镇祥云路丰瀛汽车园 → 云南省大理白族自治州大理市凤仪镇祥云路丰赢汽车园</t>
         </is>
       </c>
     </row>
@@ -14465,17 +14465,17 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>内蒙古</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车鄂尔多斯天骄路销售服务中心</t>
+          <t>小鹏汽车葫芦岛文兴路销售服务中心</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -14485,29 +14485,29 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>内蒙古鄂尔多斯市东胜区原和平宴会城北墙底商小鹏汽车交付中心 → 鄂尔多斯市康巴什区碳中和研究院内小鹏汽车</t>
+          <t>辽宁省葫芦岛市龙港区文兴路40-1号 → 辽宁省葫芦岛市龙港区龙程路</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>贵州</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>贵州华星名仕汽车销售服务有限公司</t>
+          <t>小鹏汽车杭州西溪销售服务中心</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -14517,7 +14517,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>贵州省贵阳市花溪区孟关乡红星路 13 号 10 号楼 → 贵州省贵阳市花溪区孟关苗族布依族乡福雷路2号一汽奥迪4S店</t>
+          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
         </is>
       </c>
     </row>
@@ -14529,17 +14529,17 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>山东</t>
+          <t>甘肃</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
+          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
+          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
         </is>
       </c>
     </row>
@@ -14561,17 +14561,17 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
+          <t>小鹏汽车昆明世博园销售服务中心</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
+          <t>云南省昆明市盘龙区青云街道白龙路522号 → 云南省昆明市盘龙区白龙路522号</t>
         </is>
       </c>
     </row>
@@ -14593,17 +14593,17 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>江苏</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车靖江吾悦广场销售展厅</t>
+          <t>小鹏汽车绍兴袍江汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -14613,7 +14613,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>江苏省泰州市靖江市工农路118号吾悦广场A座2号门 → 江苏省泰州市靖江市手拉手汽车小镇5号楼1层</t>
+          <t>绍兴市越城区康宁东路17号 → 浙江省绍兴市越城区康宁东路17号</t>
         </is>
       </c>
     </row>
@@ -14630,12 +14630,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车北京亦庄销售服务中心</t>
+          <t>小鹏汽车北京成寿寺销售服务中心</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -14645,7 +14645,7 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>北京市经济技术开发区科创三街15号A1幢 → 北京经济技术开发区双羊路15号</t>
+          <t>北京市朝阳区成寿寺路133号 → 北京市朝阳区小红门乡成寿寺路133号</t>
         </is>
       </c>
     </row>
@@ -14657,17 +14657,17 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>甘肃</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车张掖绿舟汽车城销售中心</t>
+          <t>小鹏汽车湖州蜀山路销售服务中心</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>甘肃省张掖市甘州区新墩镇滨河新区腾飞路与崇业路交汇处绿舟汽车城2号综合楼1层 → 甘肃省张掖市甘州区绿舟汽车城内2号楼</t>
+          <t>湖州市吴兴区蜀山路2999号 → 浙江省湖州市吴兴区蜀山路2999号</t>
         </is>
       </c>
     </row>
@@ -14689,17 +14689,17 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车昆明车行天下服务中心</t>
+          <t>小鹏汽车杭州滨康路销售服务中心</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -14709,14 +14709,14 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>云南省昆明市盘龙区新东集A座2楼小鹏汽车 → 云南省昆明市盘龙区车行天下2期新东集A座B1层</t>
+          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
@@ -14726,12 +14726,12 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车舟山甬东汽车城销售服务中心</t>
+          <t>小米之家浙江省金华市婺城区世贸城市广场汽车体验店</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>浙江省舟山市定海区经济开发区B区弘生大道466号 → 浙江省舟山市定海区临城街道经济开发区B区弘生大道466号-1</t>
+          <t>李渔路888号 → 城北街道世贸购物广场</t>
         </is>
       </c>
     </row>
@@ -14753,17 +14753,17 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>湖北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
+          <t>小鹏汽车成都锦江服务中心</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -14773,7 +14773,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
+          <t>锦丰三路77号E-5栋1层2号 → 成都市锦江区锦丰三路77号E-5栋1层2层</t>
         </is>
       </c>
     </row>
@@ -14785,17 +14785,17 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>重庆</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车榆林青云路销售服务中心</t>
+          <t>小鹏汽车重庆涪陵迎宾大道销售服务中心</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -14805,7 +14805,7 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
+          <t>重庆市涪陵区迎宾大道7号互邦涪陵汽车城 → 重庆市涪陵区迎宾大道7号互邦涪陵汽车城（东风悦达汽车4S店场地）</t>
         </is>
       </c>
     </row>
@@ -14817,17 +14817,17 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车玉溪太极路销售服务中心</t>
+          <t>小鹏汽车榆林青云路销售服务中心</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -14837,7 +14837,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>云南省玉溪市太极路103号 → 云南省玉溪市红塔区太极路103号（名爵4S店旁）</t>
+          <t>陕西省榆林市榆阳区产业四路与青云二路交汇处 → 榆阳区产业四路与青云二路交汇处</t>
         </is>
       </c>
     </row>
@@ -14849,17 +14849,17 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>江苏</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车安阳豫北汽车城销售服务中心</t>
+          <t>小鹏汽车扬州国际汽车城服务中心</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -14869,7 +14869,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>河南省安阳市安阳县弦歌大道与光明路交叉口西南角 → 河南省安阳市安阳县弦歌大道与光明路交叉口向南150米路东，小鹏汽车安阳豫北汽车城店</t>
+          <t>扬州市邗江区名车路8号 → 中国江苏省扬州市邗江区名车路8号</t>
         </is>
       </c>
     </row>
@@ -14881,17 +14881,17 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>河南</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车洛阳牡丹大道销售服务中心</t>
+          <t>小鹏汽车海宁城北销售服务中心</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -14901,7 +14901,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北新能源汽车城内 → 河南省洛阳市洛龙区牡丹大道与杜预街交叉路口西200米路北</t>
+          <t>海昌街道海宁经济技术开发区文苑路483号-1 → 浙江省海宁市海昌街道海宁经济技术开发区文苑路483号-1</t>
         </is>
       </c>
     </row>
@@ -14913,17 +14913,17 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>海南</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车资阳清巍汽车城销售服务中心</t>
+          <t>小鹏汽车海口琼山大道销售服务中心</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>四川省资阳市雁江区城东新区迎宾大道中段3号清巍汽车城（遂资眉高速出口1公里） → 四川省资阳市雁江区沱东新区迎宾大道中段 3 号</t>
+          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
         </is>
       </c>
     </row>
@@ -14945,17 +14945,17 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>江西</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车深圳光明汽车城销售服务中心</t>
+          <t>小鹏汽车吉安城北文峰汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>深圳市光明新区公明街道油麻岗路73号光明国际汽车城25#及26# → 深圳光明新区公明街道油麻岗路73号光明国际汽车城25#及26#</t>
+          <t>江西省吉安市吉安北大道122号 → 吉安市吉安北大道122号</t>
         </is>
       </c>
     </row>
@@ -14977,17 +14977,17 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>陕西</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车衢州浙西汽车城销售服务中心</t>
+          <t>小鹏汽车咸阳北上召汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>浙江省衢州市柯城区浙西大道109号16区1幢 → 浙江省衢州市柯城区浙西大道109号16区1栋</t>
+          <t>陕西省咸阳市秦皇北路秦楚汽车城商管中心1层东、西展厅 → 陕西省咸阳市秦皇北路秦楚汽车城商管中心1层</t>
         </is>
       </c>
     </row>
@@ -15009,17 +15009,17 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>辽宁</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
+          <t>小鹏汽车济南经十西路销售服务中心</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
+          <t>山东省济南市槐荫区腊山街道经十西路2800号2 幢 → 山东省济南市槐荫区腊山街道经十西路2800号</t>
         </is>
       </c>
     </row>
@@ -15041,17 +15041,17 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>陕西</t>
+          <t>云南</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车西安浐灞销售服务中心</t>
+          <t>小鹏汽车临沧南亚销售展厅</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>西安市浐灞新区汽车工业园11号 → 陕西省西安市灞桥区东三环浐灞汽车工业园11号</t>
+          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
         </is>
       </c>
     </row>
@@ -15073,17 +15073,17 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>江西</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车南昌青山湖销售服务中心</t>
+          <t>小鹏汽车新乡国际汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -15093,7 +15093,7 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>江西省南昌市青山湖区京东南大道366号 → 南昌市青山湖区京东南大道366号</t>
+          <t>河南省新乡市新飞大道南段朗公庙镇107国际汽车园内46号楼9-13展厅-小鹏汽车4S店 → 河南省新乡市高新区朗公庙镇新飞大道南段107国际汽车园内46号楼10-13号展厅</t>
         </is>
       </c>
     </row>
@@ -15105,17 +15105,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>山东</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州滨康路销售服务中心</t>
+          <t>小鹏汽车东营郝家汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -15125,7 +15125,7 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>杭州市滨江区江陵路88号 → 浙江省杭州市滨江区江陵路88号</t>
+          <t>山东省东营市垦利区北二路郝家工业园小鹏汽车 → 山东省东营市垦利区董集镇北二路14号</t>
         </is>
       </c>
     </row>
@@ -15137,17 +15137,17 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都空港销售服务中心</t>
+          <t>小鹏汽车诸暨北二环销售服务中心</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市双流区成双大道南段566号 → 成都市双流区成双大道南段566号</t>
+          <t>浙江省绍兴市诸暨市陶朱街道北二环路9号 → 浙江省绍兴市诸暨市陶朱街道北二环路9号1幢1楼</t>
         </is>
       </c>
     </row>
@@ -15169,17 +15169,17 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河南</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车杭州西溪销售服务中心</t>
+          <t>小鹏汽车许昌许州北路销售服务中心</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -15189,7 +15189,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>杭州市西湖区西溪路698号一层-2 → 杭州市西湖区西溪路698 号一层-2</t>
+          <t>河南省许昌市建安区许州路与新东街交叉口正通汽贸城内 → 河南省许昌市许州路与新东街交叉口正通汽贸城内</t>
         </is>
       </c>
     </row>
@@ -15201,17 +15201,17 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车成都龙潭寺销售服务中心</t>
+          <t>小鹏汽车温州瓯海国际汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -15221,7 +15221,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>四川省成都市成华区华泰路76号 → 成都市成华区华泰路76号</t>
+          <t>温州市瓯海区娄桥街道瓯融汽车产业园1号 → 浙江省温州市瓯海区永庆街瓯融汽车产业园1号</t>
         </is>
       </c>
     </row>
@@ -15238,12 +15238,12 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车佛山顺德陈村销售服务中心</t>
+          <t>小鹏汽车云浮环市西路销售服务中心</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一小鹏汽车佛山顺德陈村销售服务中心 → 广东省佛山市顺德区陈村镇南涌居委会芸香围105国道边30号之一</t>
+          <t>云浮市云城区环市西路循常村委路口处（中裕云成二手车交易市场左侧） → 云浮市云城区环市西路循常村委路口处（恒大城南侧）</t>
         </is>
       </c>
     </row>
@@ -15265,17 +15265,17 @@
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>云南</t>
+          <t>湖北</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车临沧南亚销售展厅</t>
+          <t>小鹏汽车随州鹿鹤大道销售服务中心</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -15285,7 +15285,7 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>云南省临沧市临翔区忙畔街道办事处文伟佳村委会南亚汽车主题园3栋1-2室 → 临沧市临翔区缅宁大道214南亚汽车主题园内</t>
+          <t>随州鹿鹤大道28号 → 湖北省随州市高新区鹿鹤大道28号1-3层101号1层</t>
         </is>
       </c>
     </row>
@@ -15297,17 +15297,17 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车岳阳巴陵东路销售服务中心</t>
+          <t>小鹏汽车达州杨柳汽车园销售服务中心</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -15317,7 +15317,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>岳阳市巴陵东路382号 → 湖南省岳阳市岳阳楼区通海路管理处巴陵东路382号</t>
+          <t>达州市达川区杨柳街道柳林路13号 → 四川省达州市达川区杨柳街道柳林路13号</t>
         </is>
       </c>
     </row>
@@ -15329,17 +15329,17 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>海南</t>
+          <t>安徽</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车海口琼山大道销售服务中心</t>
+          <t>小鹏汽车合肥包河汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -15349,7 +15349,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>海口市美兰区琼山大道260号 → 海南省海口市美兰区琼山大道260号</t>
+          <t>安徽省合肥市包河经济开发区繁华大道29华天大厦向东20米3号整栋标准厂房 → 繁华大道29华天大厦向东20米3号整栋标准厂房</t>
         </is>
       </c>
     </row>
@@ -15361,17 +15361,17 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>重庆</t>
+          <t>辽宁</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车重庆礼嘉服务中心</t>
+          <t>小鹏汽车大连华北路汽车城销售服务中心</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>重庆市两江新区礼环北路10号普洛斯（重庆）物流园2期礼嘉园区B3栋小鹏汽车 → 重庆市两江新区礼洁路10号</t>
+          <t>辽宁省大连市甘井子区华北路北市商贸街158号7号 → :辽宁省大连市甘井子区华北路北市商贸街158号</t>
         </is>
       </c>
     </row>
@@ -15420,22 +15420,22 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>小鹏</t>
+          <t>奥迪</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>黑龙江</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩二环北路销售中心</t>
+          <t>牡丹江中信恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
+          <t>牡丹江中源恒业汽车销售服务有限公司</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -15457,17 +15457,17 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>河北</t>
+          <t>四川</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃维修中心（过渡运营）</t>
+          <t>乐山天牛华韵4S中心</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>唐山申联凯沃4S中心（过渡运营）</t>
+          <t>乐山天牛华韵维修中心</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -15516,22 +15516,22 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小米</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>四川</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵4S中心</t>
+          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>乐山天牛华韵维修中心</t>
+          <t>小米汽车浙江宁波市宁海县西子国际</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -15548,22 +15548,22 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>小米</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>河北</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波宁海县西子国际购物中心</t>
+          <t>唐山申联凯沃维修中心（过渡运营）</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>小米汽车浙江宁波市宁海县西子国际</t>
+          <t>唐山申联凯沃4S中心（过渡运营）</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -15580,22 +15580,22 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>沃尔沃</t>
+          <t>小鹏</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>广东</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>深圳德利行光明卫星店</t>
+          <t>小鹏汽车台州黄岩二环北路销售中心</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>深圳深标嘉光明卫星店</t>
+          <t>小鹏汽车台州黄岩手拉手汽车广场销售中心</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -15612,22 +15612,22 @@
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>奥迪</t>
+          <t>沃尔沃</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>黑龙江</t>
+          <t>广东</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中信恒业汽车销售服务有限公司</t>
+          <t>深圳德利行光明卫星店</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>牡丹江中源恒业汽车销售服务有限公司</t>
+          <t>深圳深标嘉光明卫星店</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">

</xml_diff>